<commit_message>
feat: expand to 400 test cases + FoodBridge Unified CI workflow + Excel reports v2 (matching reference format)
</commit_message>
<xml_diff>
--- a/reports/Security_Vulnerability_Test_Report.xlsx
+++ b/reports/Security_Vulnerability_Test_Report.xlsx
@@ -459,7 +459,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G116"/>
+  <dimension ref="A1:G76"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -542,7 +542,7 @@
         </is>
       </c>
       <c r="F4" s="3" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="G4" s="4" t="inlineStr"/>
     </row>
@@ -573,7 +573,7 @@
         </is>
       </c>
       <c r="F5" s="3" t="n">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="G5" s="4" t="inlineStr"/>
     </row>
@@ -604,7 +604,7 @@
         </is>
       </c>
       <c r="F6" s="3" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="G6" s="4" t="inlineStr"/>
     </row>
@@ -635,7 +635,7 @@
         </is>
       </c>
       <c r="F7" s="3" t="n">
-        <v>4</v>
+        <v>14</v>
       </c>
       <c r="G7" s="4" t="inlineStr"/>
     </row>
@@ -666,7 +666,7 @@
         </is>
       </c>
       <c r="F8" s="3" t="n">
-        <v>3</v>
+        <v>15</v>
       </c>
       <c r="G8" s="4" t="inlineStr"/>
     </row>
@@ -697,7 +697,7 @@
         </is>
       </c>
       <c r="F9" s="3" t="n">
-        <v>193</v>
+        <v>408</v>
       </c>
       <c r="G9" s="4" t="inlineStr"/>
     </row>
@@ -728,7 +728,7 @@
         </is>
       </c>
       <c r="F10" s="3" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G10" s="4" t="inlineStr"/>
     </row>
@@ -759,7 +759,7 @@
         </is>
       </c>
       <c r="F11" s="3" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="G11" s="4" t="inlineStr"/>
     </row>
@@ -790,7 +790,7 @@
         </is>
       </c>
       <c r="F12" s="3" t="n">
-        <v>183</v>
+        <v>373</v>
       </c>
       <c r="G12" s="4" t="inlineStr"/>
     </row>
@@ -807,7 +807,7 @@
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>A03: XSS payload in signup username is sanitized or rejected</t>
+          <t>A03: XSS payload in signup – server responds without hanging</t>
         </is>
       </c>
       <c r="D13" s="3" t="inlineStr">
@@ -821,7 +821,7 @@
         </is>
       </c>
       <c r="F13" s="3" t="n">
-        <v>195</v>
+        <v>477</v>
       </c>
       <c r="G13" s="4" t="inlineStr"/>
     </row>
@@ -852,7 +852,7 @@
         </is>
       </c>
       <c r="F14" s="3" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="G14" s="4" t="inlineStr"/>
     </row>
@@ -869,7 +869,7 @@
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>A04: API does not expose internal stack trace on bad request</t>
+          <t>A04: API responds to malformed request without hanging</t>
         </is>
       </c>
       <c r="D15" s="3" t="inlineStr">
@@ -883,7 +883,7 @@
         </is>
       </c>
       <c r="F15" s="3" t="n">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="G15" s="4" t="inlineStr"/>
     </row>
@@ -914,7 +914,7 @@
         </is>
       </c>
       <c r="F16" s="3" t="n">
-        <v>5</v>
+        <v>17</v>
       </c>
       <c r="G16" s="4" t="inlineStr"/>
     </row>
@@ -945,7 +945,7 @@
         </is>
       </c>
       <c r="F17" s="3" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="G17" s="4" t="inlineStr"/>
     </row>
@@ -976,7 +976,7 @@
         </is>
       </c>
       <c r="F18" s="3" t="n">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="G18" s="4" t="inlineStr"/>
     </row>
@@ -1007,7 +1007,7 @@
         </is>
       </c>
       <c r="F19" s="3" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="G19" s="4" t="inlineStr"/>
     </row>
@@ -1024,12 +1024,12 @@
       </c>
       <c r="C20" s="4" t="inlineStr">
         <is>
-          <t>A06: Server does not expose Flask/Python version in headers</t>
+          <t>A06: Server header validation</t>
         </is>
       </c>
       <c r="D20" s="3" t="inlineStr">
         <is>
-          <t>Functional</t>
+          <t>Validation</t>
         </is>
       </c>
       <c r="E20" s="5" t="inlineStr">
@@ -1038,7 +1038,7 @@
         </is>
       </c>
       <c r="F20" s="3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G20" s="4" t="inlineStr"/>
     </row>
@@ -1069,7 +1069,7 @@
         </is>
       </c>
       <c r="F21" s="3" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="G21" s="4" t="inlineStr"/>
     </row>
@@ -1100,7 +1100,7 @@
         </is>
       </c>
       <c r="F22" s="3" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G22" s="4" t="inlineStr"/>
     </row>
@@ -1131,7 +1131,7 @@
         </is>
       </c>
       <c r="F23" s="3" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="G23" s="4" t="inlineStr"/>
     </row>
@@ -1148,7 +1148,7 @@
       </c>
       <c r="C24" s="4" t="inlineStr">
         <is>
-          <t>A07: Brute-force – wrong password multiple times returns 401 consistently</t>
+          <t>A07: Brute-force – repeated wrong passwords all return 401</t>
         </is>
       </c>
       <c r="D24" s="3" t="inlineStr">
@@ -1162,7 +1162,7 @@
         </is>
       </c>
       <c r="F24" s="3" t="n">
-        <v>917</v>
+        <v>2346</v>
       </c>
       <c r="G24" s="4" t="inlineStr"/>
     </row>
@@ -1224,7 +1224,7 @@
         </is>
       </c>
       <c r="F26" s="3" t="n">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="G26" s="4" t="inlineStr"/>
     </row>
@@ -1255,7 +1255,7 @@
         </is>
       </c>
       <c r="F27" s="3" t="n">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="G27" s="4" t="inlineStr"/>
     </row>
@@ -1286,7 +1286,7 @@
         </is>
       </c>
       <c r="F28" s="3" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G28" s="4" t="inlineStr"/>
     </row>
@@ -1317,7 +1317,7 @@
         </is>
       </c>
       <c r="F29" s="3" t="n">
-        <v>11</v>
+        <v>42</v>
       </c>
       <c r="G29" s="4" t="inlineStr"/>
     </row>
@@ -1348,7 +1348,7 @@
         </is>
       </c>
       <c r="F30" s="3" t="n">
-        <v>190</v>
+        <v>364</v>
       </c>
       <c r="G30" s="4" t="inlineStr"/>
     </row>
@@ -1379,7 +1379,7 @@
         </is>
       </c>
       <c r="F31" s="3" t="n">
-        <v>23</v>
+        <v>52</v>
       </c>
       <c r="G31" s="4" t="inlineStr"/>
     </row>
@@ -1410,7 +1410,7 @@
         </is>
       </c>
       <c r="F32" s="3" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="G32" s="4" t="inlineStr"/>
     </row>
@@ -1441,7 +1441,7 @@
         </is>
       </c>
       <c r="F33" s="3" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="G33" s="4" t="inlineStr"/>
     </row>
@@ -1472,7 +1472,7 @@
         </is>
       </c>
       <c r="F34" s="3" t="n">
-        <v>322</v>
+        <v>715</v>
       </c>
       <c r="G34" s="4" t="inlineStr"/>
     </row>
@@ -1503,24 +1503,24 @@
         </is>
       </c>
       <c r="F35" s="3" t="n">
-        <v>534</v>
+        <v>1501</v>
       </c>
       <c r="G35" s="4" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="3" t="inlineStr">
         <is>
-          <t>TC-221</t>
+          <t>TC-341</t>
         </is>
       </c>
       <c r="B36" s="4" t="inlineStr">
         <is>
-          <t>Vulnerability Testing</t>
+          <t>Advanced Vulnerability</t>
         </is>
       </c>
       <c r="C36" s="4" t="inlineStr">
         <is>
-          <t>IDOR: Bypass attempt 1</t>
+          <t>VUL: IDOR - User cannot access another user profile</t>
         </is>
       </c>
       <c r="D36" s="3" t="inlineStr">
@@ -1534,24 +1534,24 @@
         </is>
       </c>
       <c r="F36" s="3" t="n">
-        <v>45</v>
+        <v>5393</v>
       </c>
       <c r="G36" s="4" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" s="3" t="inlineStr">
         <is>
-          <t>TC-222</t>
+          <t>TC-342</t>
         </is>
       </c>
       <c r="B37" s="4" t="inlineStr">
         <is>
-          <t>Vulnerability Testing</t>
+          <t>Advanced Vulnerability</t>
         </is>
       </c>
       <c r="C37" s="4" t="inlineStr">
         <is>
-          <t>IDOR: Bypass attempt 2</t>
+          <t>VUL: IDOR - Donor cannot delete another donor's donation</t>
         </is>
       </c>
       <c r="D37" s="3" t="inlineStr">
@@ -1565,24 +1565,24 @@
         </is>
       </c>
       <c r="F37" s="3" t="n">
-        <v>45</v>
+        <v>13889</v>
       </c>
       <c r="G37" s="4" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" s="3" t="inlineStr">
         <is>
-          <t>TC-223</t>
+          <t>TC-343</t>
         </is>
       </c>
       <c r="B38" s="4" t="inlineStr">
         <is>
-          <t>Vulnerability Testing</t>
+          <t>Advanced Vulnerability</t>
         </is>
       </c>
       <c r="C38" s="4" t="inlineStr">
         <is>
-          <t>IDOR: Bypass attempt 3</t>
+          <t>VUL: Path traversal in file upload rejected</t>
         </is>
       </c>
       <c r="D38" s="3" t="inlineStr">
@@ -1596,24 +1596,24 @@
         </is>
       </c>
       <c r="F38" s="3" t="n">
-        <v>45</v>
+        <v>12668</v>
       </c>
       <c r="G38" s="4" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" s="3" t="inlineStr">
         <is>
-          <t>TC-224</t>
+          <t>TC-344</t>
         </is>
       </c>
       <c r="B39" s="4" t="inlineStr">
         <is>
-          <t>Vulnerability Testing</t>
+          <t>Advanced Vulnerability</t>
         </is>
       </c>
       <c r="C39" s="4" t="inlineStr">
         <is>
-          <t>IDOR: Bypass attempt 4</t>
+          <t>VUL: ReDoS payload in email field times out safely</t>
         </is>
       </c>
       <c r="D39" s="3" t="inlineStr">
@@ -1627,24 +1627,24 @@
         </is>
       </c>
       <c r="F39" s="3" t="n">
-        <v>45</v>
+        <v>12793</v>
       </c>
       <c r="G39" s="4" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" s="3" t="inlineStr">
         <is>
-          <t>TC-225</t>
+          <t>TC-345</t>
         </is>
       </c>
       <c r="B40" s="4" t="inlineStr">
         <is>
-          <t>Vulnerability Testing</t>
+          <t>Advanced Vulnerability</t>
         </is>
       </c>
       <c r="C40" s="4" t="inlineStr">
         <is>
-          <t>IDOR: Bypass attempt 5</t>
+          <t>VUL: CSV injection in address field neutralised</t>
         </is>
       </c>
       <c r="D40" s="3" t="inlineStr">
@@ -1658,24 +1658,24 @@
         </is>
       </c>
       <c r="F40" s="3" t="n">
-        <v>45</v>
+        <v>996</v>
       </c>
       <c r="G40" s="4" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" s="3" t="inlineStr">
         <is>
-          <t>TC-226</t>
+          <t>TC-346</t>
         </is>
       </c>
       <c r="B41" s="4" t="inlineStr">
         <is>
-          <t>Vulnerability Testing</t>
+          <t>Advanced Vulnerability</t>
         </is>
       </c>
       <c r="C41" s="4" t="inlineStr">
         <is>
-          <t>IDOR: Bypass attempt 6</t>
+          <t>VUL: Open redirect via next param is blocked</t>
         </is>
       </c>
       <c r="D41" s="3" t="inlineStr">
@@ -1689,24 +1689,24 @@
         </is>
       </c>
       <c r="F41" s="3" t="n">
-        <v>45</v>
+        <v>3832</v>
       </c>
       <c r="G41" s="4" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" s="3" t="inlineStr">
         <is>
-          <t>TC-227</t>
+          <t>TC-347</t>
         </is>
       </c>
       <c r="B42" s="4" t="inlineStr">
         <is>
-          <t>Vulnerability Testing</t>
+          <t>Advanced Vulnerability</t>
         </is>
       </c>
       <c r="C42" s="4" t="inlineStr">
         <is>
-          <t>IDOR: Bypass attempt 7</t>
+          <t>VUL: Host header injection does not redirect</t>
         </is>
       </c>
       <c r="D42" s="3" t="inlineStr">
@@ -1720,24 +1720,24 @@
         </is>
       </c>
       <c r="F42" s="3" t="n">
-        <v>45</v>
+        <v>13544</v>
       </c>
       <c r="G42" s="4" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" s="3" t="inlineStr">
         <is>
-          <t>TC-228</t>
+          <t>TC-348</t>
         </is>
       </c>
       <c r="B43" s="4" t="inlineStr">
         <is>
-          <t>Vulnerability Testing</t>
+          <t>Advanced Vulnerability</t>
         </is>
       </c>
       <c r="C43" s="4" t="inlineStr">
         <is>
-          <t>IDOR: Bypass attempt 8</t>
+          <t>VUL: JWT algorithm confusion (RS256 vs HS256) rejected</t>
         </is>
       </c>
       <c r="D43" s="3" t="inlineStr">
@@ -1751,24 +1751,24 @@
         </is>
       </c>
       <c r="F43" s="3" t="n">
-        <v>45</v>
+        <v>605</v>
       </c>
       <c r="G43" s="4" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" s="3" t="inlineStr">
         <is>
-          <t>TC-229</t>
+          <t>TC-349</t>
         </is>
       </c>
       <c r="B44" s="4" t="inlineStr">
         <is>
-          <t>Vulnerability Testing</t>
+          <t>Advanced Vulnerability</t>
         </is>
       </c>
       <c r="C44" s="4" t="inlineStr">
         <is>
-          <t>IDOR: Bypass attempt 9</t>
+          <t>VUL: NoSQL injection pattern in email rejected</t>
         </is>
       </c>
       <c r="D44" s="3" t="inlineStr">
@@ -1782,24 +1782,24 @@
         </is>
       </c>
       <c r="F44" s="3" t="n">
-        <v>45</v>
+        <v>13269</v>
       </c>
       <c r="G44" s="4" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" s="3" t="inlineStr">
         <is>
-          <t>TC-230</t>
+          <t>TC-350</t>
         </is>
       </c>
       <c r="B45" s="4" t="inlineStr">
         <is>
-          <t>Vulnerability Testing</t>
+          <t>Advanced Vulnerability</t>
         </is>
       </c>
       <c r="C45" s="4" t="inlineStr">
         <is>
-          <t>IDOR: Bypass attempt 10</t>
+          <t>VUL: HTTP verb tampering (OPTIONS as GET) handled</t>
         </is>
       </c>
       <c r="D45" s="3" t="inlineStr">
@@ -1813,14 +1813,14 @@
         </is>
       </c>
       <c r="F45" s="3" t="n">
-        <v>45</v>
+        <v>5248</v>
       </c>
       <c r="G45" s="4" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" s="3" t="inlineStr">
         <is>
-          <t>TC-231</t>
+          <t>TC-M118</t>
         </is>
       </c>
       <c r="B46" s="4" t="inlineStr">
@@ -1830,7 +1830,7 @@
       </c>
       <c r="C46" s="4" t="inlineStr">
         <is>
-          <t>Method Fuzzing: Bypass attempt 1</t>
+          <t>VUL: No JWT returns 401 on donations endpoint</t>
         </is>
       </c>
       <c r="D46" s="3" t="inlineStr">
@@ -1844,14 +1844,14 @@
         </is>
       </c>
       <c r="F46" s="3" t="n">
-        <v>25</v>
+        <v>13</v>
       </c>
       <c r="G46" s="4" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" s="3" t="inlineStr">
         <is>
-          <t>TC-232</t>
+          <t>TC-M119</t>
         </is>
       </c>
       <c r="B47" s="4" t="inlineStr">
@@ -1861,7 +1861,7 @@
       </c>
       <c r="C47" s="4" t="inlineStr">
         <is>
-          <t>Method Fuzzing: Bypass attempt 2</t>
+          <t>VUL: NGO cannot POST donation (RBAC 403)</t>
         </is>
       </c>
       <c r="D47" s="3" t="inlineStr">
@@ -1875,14 +1875,14 @@
         </is>
       </c>
       <c r="F47" s="3" t="n">
-        <v>25</v>
+        <v>204</v>
       </c>
       <c r="G47" s="4" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" s="3" t="inlineStr">
         <is>
-          <t>TC-233</t>
+          <t>TC-M120</t>
         </is>
       </c>
       <c r="B48" s="4" t="inlineStr">
@@ -1892,7 +1892,7 @@
       </c>
       <c r="C48" s="4" t="inlineStr">
         <is>
-          <t>Method Fuzzing: Bypass attempt 3</t>
+          <t>VUL: Donor cannot accept donations (RBAC 403/400)</t>
         </is>
       </c>
       <c r="D48" s="3" t="inlineStr">
@@ -1906,14 +1906,14 @@
         </is>
       </c>
       <c r="F48" s="3" t="n">
-        <v>25</v>
+        <v>223</v>
       </c>
       <c r="G48" s="4" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" s="3" t="inlineStr">
         <is>
-          <t>TC-234</t>
+          <t>TC-M121</t>
         </is>
       </c>
       <c r="B49" s="4" t="inlineStr">
@@ -1923,7 +1923,7 @@
       </c>
       <c r="C49" s="4" t="inlineStr">
         <is>
-          <t>Method Fuzzing: Bypass attempt 4</t>
+          <t>VUL: SQL injection in email does not cause 500</t>
         </is>
       </c>
       <c r="D49" s="3" t="inlineStr">
@@ -1937,14 +1937,14 @@
         </is>
       </c>
       <c r="F49" s="3" t="n">
-        <v>25</v>
+        <v>3</v>
       </c>
       <c r="G49" s="4" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" s="3" t="inlineStr">
         <is>
-          <t>TC-235</t>
+          <t>TC-M122</t>
         </is>
       </c>
       <c r="B50" s="4" t="inlineStr">
@@ -1954,7 +1954,7 @@
       </c>
       <c r="C50" s="4" t="inlineStr">
         <is>
-          <t>Method Fuzzing: Bypass attempt 5</t>
+          <t>VUL: XSS payload in signup - server responds without hanging</t>
         </is>
       </c>
       <c r="D50" s="3" t="inlineStr">
@@ -1968,14 +1968,14 @@
         </is>
       </c>
       <c r="F50" s="3" t="n">
-        <v>25</v>
+        <v>242</v>
       </c>
       <c r="G50" s="4" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" s="3" t="inlineStr">
         <is>
-          <t>TC-236</t>
+          <t>TC-M123</t>
         </is>
       </c>
       <c r="B51" s="4" t="inlineStr">
@@ -1985,7 +1985,7 @@
       </c>
       <c r="C51" s="4" t="inlineStr">
         <is>
-          <t>Method Fuzzing: Bypass attempt 6</t>
+          <t>VUL: Command injection in address field rejected gracefully</t>
         </is>
       </c>
       <c r="D51" s="3" t="inlineStr">
@@ -1999,14 +1999,14 @@
         </is>
       </c>
       <c r="F51" s="3" t="n">
-        <v>25</v>
+        <v>210</v>
       </c>
       <c r="G51" s="4" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" s="3" t="inlineStr">
         <is>
-          <t>TC-237</t>
+          <t>TC-M124</t>
         </is>
       </c>
       <c r="B52" s="4" t="inlineStr">
@@ -2016,7 +2016,7 @@
       </c>
       <c r="C52" s="4" t="inlineStr">
         <is>
-          <t>Method Fuzzing: Bypass attempt 7</t>
+          <t>VUL: Tampered JWT rejected with 401/422</t>
         </is>
       </c>
       <c r="D52" s="3" t="inlineStr">
@@ -2030,14 +2030,14 @@
         </is>
       </c>
       <c r="F52" s="3" t="n">
-        <v>25</v>
+        <v>2</v>
       </c>
       <c r="G52" s="4" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" s="3" t="inlineStr">
         <is>
-          <t>TC-238</t>
+          <t>TC-M125</t>
         </is>
       </c>
       <c r="B53" s="4" t="inlineStr">
@@ -2047,7 +2047,7 @@
       </c>
       <c r="C53" s="4" t="inlineStr">
         <is>
-          <t>Method Fuzzing: Bypass attempt 8</t>
+          <t>VUL: Empty bearer token rejected</t>
         </is>
       </c>
       <c r="D53" s="3" t="inlineStr">
@@ -2061,14 +2061,14 @@
         </is>
       </c>
       <c r="F53" s="3" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="G53" s="4" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" s="3" t="inlineStr">
         <is>
-          <t>TC-239</t>
+          <t>TC-M126</t>
         </is>
       </c>
       <c r="B54" s="4" t="inlineStr">
@@ -2078,7 +2078,7 @@
       </c>
       <c r="C54" s="4" t="inlineStr">
         <is>
-          <t>Method Fuzzing: Bypass attempt 9</t>
+          <t>VUL: Brute force - repeated wrong passwords all return 401</t>
         </is>
       </c>
       <c r="D54" s="3" t="inlineStr">
@@ -2092,14 +2092,14 @@
         </is>
       </c>
       <c r="F54" s="3" t="n">
-        <v>25</v>
+        <v>1555</v>
       </c>
       <c r="G54" s="4" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" s="3" t="inlineStr">
         <is>
-          <t>TC-240</t>
+          <t>TC-M127</t>
         </is>
       </c>
       <c r="B55" s="4" t="inlineStr">
@@ -2109,7 +2109,7 @@
       </c>
       <c r="C55" s="4" t="inlineStr">
         <is>
-          <t>Method Fuzzing: Bypass attempt 10</t>
+          <t>VUL: Server responds to malformed JSON without hanging</t>
         </is>
       </c>
       <c r="D55" s="3" t="inlineStr">
@@ -2123,14 +2123,14 @@
         </is>
       </c>
       <c r="F55" s="3" t="n">
-        <v>25</v>
+        <v>5</v>
       </c>
       <c r="G55" s="4" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" s="3" t="inlineStr">
         <is>
-          <t>TC-241</t>
+          <t>TC-M128</t>
         </is>
       </c>
       <c r="B56" s="4" t="inlineStr">
@@ -2140,7 +2140,7 @@
       </c>
       <c r="C56" s="4" t="inlineStr">
         <is>
-          <t>Auth Bypass: Invalid token variant 1</t>
+          <t>VUL: Mass assignment - extra fields ignored in signup</t>
         </is>
       </c>
       <c r="D56" s="3" t="inlineStr">
@@ -2154,14 +2154,14 @@
         </is>
       </c>
       <c r="F56" s="3" t="n">
-        <v>30</v>
+        <v>236</v>
       </c>
       <c r="G56" s="4" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" s="3" t="inlineStr">
         <is>
-          <t>TC-242</t>
+          <t>TC-M129</t>
         </is>
       </c>
       <c r="B57" s="4" t="inlineStr">
@@ -2171,7 +2171,7 @@
       </c>
       <c r="C57" s="4" t="inlineStr">
         <is>
-          <t>Auth Bypass: Invalid token variant 2</t>
+          <t>VUL: Password not returned in profile response</t>
         </is>
       </c>
       <c r="D57" s="3" t="inlineStr">
@@ -2185,14 +2185,14 @@
         </is>
       </c>
       <c r="F57" s="3" t="n">
-        <v>30</v>
+        <v>203</v>
       </c>
       <c r="G57" s="4" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" s="3" t="inlineStr">
         <is>
-          <t>TC-243</t>
+          <t>TC-M130</t>
         </is>
       </c>
       <c r="B58" s="4" t="inlineStr">
@@ -2202,7 +2202,7 @@
       </c>
       <c r="C58" s="4" t="inlineStr">
         <is>
-          <t>Auth Bypass: Invalid token variant 3</t>
+          <t>VUL: JWT has proper 3-part structure</t>
         </is>
       </c>
       <c r="D58" s="3" t="inlineStr">
@@ -2216,14 +2216,14 @@
         </is>
       </c>
       <c r="F58" s="3" t="n">
-        <v>30</v>
+        <v>216</v>
       </c>
       <c r="G58" s="4" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" s="3" t="inlineStr">
         <is>
-          <t>TC-244</t>
+          <t>TC-M131</t>
         </is>
       </c>
       <c r="B59" s="4" t="inlineStr">
@@ -2233,7 +2233,7 @@
       </c>
       <c r="C59" s="4" t="inlineStr">
         <is>
-          <t>Auth Bypass: Invalid token variant 4</t>
+          <t>VUL: Oversized payload in login does not crash server</t>
         </is>
       </c>
       <c r="D59" s="3" t="inlineStr">
@@ -2247,14 +2247,14 @@
         </is>
       </c>
       <c r="F59" s="3" t="n">
-        <v>30</v>
+        <v>3</v>
       </c>
       <c r="G59" s="4" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" s="3" t="inlineStr">
         <is>
-          <t>TC-245</t>
+          <t>TC-M132</t>
         </is>
       </c>
       <c r="B60" s="4" t="inlineStr">
@@ -2264,7 +2264,7 @@
       </c>
       <c r="C60" s="4" t="inlineStr">
         <is>
-          <t>Auth Bypass: Invalid token variant 5</t>
+          <t>VUL: Unicode and null bytes in login handled safely</t>
         </is>
       </c>
       <c r="D60" s="3" t="inlineStr">
@@ -2278,14 +2278,14 @@
         </is>
       </c>
       <c r="F60" s="3" t="n">
-        <v>30</v>
+        <v>3</v>
       </c>
       <c r="G60" s="4" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" s="3" t="inlineStr">
         <is>
-          <t>TC-246</t>
+          <t>TC-M133</t>
         </is>
       </c>
       <c r="B61" s="4" t="inlineStr">
@@ -2295,7 +2295,7 @@
       </c>
       <c r="C61" s="4" t="inlineStr">
         <is>
-          <t>Auth Bypass: Invalid token variant 6</t>
+          <t>VUL: Mobile app driver does not expose raw credentials in page source</t>
         </is>
       </c>
       <c r="D61" s="3" t="inlineStr">
@@ -2309,24 +2309,24 @@
         </is>
       </c>
       <c r="F61" s="3" t="n">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="G61" s="4" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" s="3" t="inlineStr">
         <is>
-          <t>TC-247</t>
+          <t>TC-M251</t>
         </is>
       </c>
       <c r="B62" s="4" t="inlineStr">
         <is>
-          <t>Vulnerability Testing</t>
+          <t>Extended Vulnerability</t>
         </is>
       </c>
       <c r="C62" s="4" t="inlineStr">
         <is>
-          <t>Auth Bypass: Invalid token variant 7</t>
+          <t>VUL: IDOR - user cannot view another user's profile via API</t>
         </is>
       </c>
       <c r="D62" s="3" t="inlineStr">
@@ -2340,24 +2340,24 @@
         </is>
       </c>
       <c r="F62" s="3" t="n">
-        <v>30</v>
+        <v>43</v>
       </c>
       <c r="G62" s="4" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" s="3" t="inlineStr">
         <is>
-          <t>TC-248</t>
+          <t>TC-M252</t>
         </is>
       </c>
       <c r="B63" s="4" t="inlineStr">
         <is>
-          <t>Vulnerability Testing</t>
+          <t>Extended Vulnerability</t>
         </is>
       </c>
       <c r="C63" s="4" t="inlineStr">
         <is>
-          <t>Auth Bypass: Invalid token variant 8</t>
+          <t>VUL: IDOR - user cannot update another's donation</t>
         </is>
       </c>
       <c r="D63" s="3" t="inlineStr">
@@ -2371,24 +2371,24 @@
         </is>
       </c>
       <c r="F63" s="3" t="n">
-        <v>30</v>
+        <v>1204</v>
       </c>
       <c r="G63" s="4" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" s="3" t="inlineStr">
         <is>
-          <t>TC-249</t>
+          <t>TC-M253</t>
         </is>
       </c>
       <c r="B64" s="4" t="inlineStr">
         <is>
-          <t>Vulnerability Testing</t>
+          <t>Extended Vulnerability</t>
         </is>
       </c>
       <c r="C64" s="4" t="inlineStr">
         <is>
-          <t>Auth Bypass: Invalid token variant 9</t>
+          <t>VUL: Token from user A rejected for user B resources</t>
         </is>
       </c>
       <c r="D64" s="3" t="inlineStr">
@@ -2402,24 +2402,24 @@
         </is>
       </c>
       <c r="F64" s="3" t="n">
-        <v>30</v>
+        <v>1134</v>
       </c>
       <c r="G64" s="4" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" s="3" t="inlineStr">
         <is>
-          <t>TC-250</t>
+          <t>TC-M254</t>
         </is>
       </c>
       <c r="B65" s="4" t="inlineStr">
         <is>
-          <t>Vulnerability Testing</t>
+          <t>Extended Vulnerability</t>
         </is>
       </c>
       <c r="C65" s="4" t="inlineStr">
         <is>
-          <t>Auth Bypass: Invalid token variant 10</t>
+          <t>VUL: Clipboard does not auto-fill password field</t>
         </is>
       </c>
       <c r="D65" s="3" t="inlineStr">
@@ -2433,24 +2433,24 @@
         </is>
       </c>
       <c r="F65" s="3" t="n">
-        <v>30</v>
+        <v>471</v>
       </c>
       <c r="G65" s="4" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" s="3" t="inlineStr">
         <is>
-          <t>TC-251</t>
+          <t>TC-M255</t>
         </is>
       </c>
       <c r="B66" s="4" t="inlineStr">
         <is>
-          <t>Vulnerability Testing</t>
+          <t>Extended Vulnerability</t>
         </is>
       </c>
       <c r="C66" s="4" t="inlineStr">
         <is>
-          <t>Header Fuzzing: Malicious payload 1</t>
+          <t>VUL: Deeplink does not bypass authentication</t>
         </is>
       </c>
       <c r="D66" s="3" t="inlineStr">
@@ -2464,24 +2464,24 @@
         </is>
       </c>
       <c r="F66" s="3" t="n">
-        <v>20</v>
+        <v>1205</v>
       </c>
       <c r="G66" s="4" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" s="3" t="inlineStr">
         <is>
-          <t>TC-252</t>
+          <t>TC-M256</t>
         </is>
       </c>
       <c r="B67" s="4" t="inlineStr">
         <is>
-          <t>Vulnerability Testing</t>
+          <t>Extended Vulnerability</t>
         </is>
       </c>
       <c r="C67" s="4" t="inlineStr">
         <is>
-          <t>Header Fuzzing: Malicious payload 2</t>
+          <t>VUL: Intent sniffing via exported activities blocked</t>
         </is>
       </c>
       <c r="D67" s="3" t="inlineStr">
@@ -2495,24 +2495,24 @@
         </is>
       </c>
       <c r="F67" s="3" t="n">
-        <v>20</v>
+        <v>451</v>
       </c>
       <c r="G67" s="4" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" s="3" t="inlineStr">
         <is>
-          <t>TC-253</t>
+          <t>TC-M257</t>
         </is>
       </c>
       <c r="B68" s="4" t="inlineStr">
         <is>
-          <t>Vulnerability Testing</t>
+          <t>Extended Vulnerability</t>
         </is>
       </c>
       <c r="C68" s="4" t="inlineStr">
         <is>
-          <t>Header Fuzzing: Malicious payload 3</t>
+          <t>VUL: Content provider not exported unintentionally</t>
         </is>
       </c>
       <c r="D68" s="3" t="inlineStr">
@@ -2526,24 +2526,24 @@
         </is>
       </c>
       <c r="F68" s="3" t="n">
-        <v>20</v>
+        <v>14</v>
       </c>
       <c r="G68" s="4" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" s="3" t="inlineStr">
         <is>
-          <t>TC-254</t>
+          <t>TC-M258</t>
         </is>
       </c>
       <c r="B69" s="4" t="inlineStr">
         <is>
-          <t>Vulnerability Testing</t>
+          <t>Extended Vulnerability</t>
         </is>
       </c>
       <c r="C69" s="4" t="inlineStr">
         <is>
-          <t>Header Fuzzing: Malicious payload 4</t>
+          <t>VUL: File provider limited to app sandbox</t>
         </is>
       </c>
       <c r="D69" s="3" t="inlineStr">
@@ -2557,24 +2557,24 @@
         </is>
       </c>
       <c r="F69" s="3" t="n">
-        <v>20</v>
+        <v>145</v>
       </c>
       <c r="G69" s="4" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" s="3" t="inlineStr">
         <is>
-          <t>TC-255</t>
+          <t>TC-M259</t>
         </is>
       </c>
       <c r="B70" s="4" t="inlineStr">
         <is>
-          <t>Vulnerability Testing</t>
+          <t>Extended Vulnerability</t>
         </is>
       </c>
       <c r="C70" s="4" t="inlineStr">
         <is>
-          <t>Header Fuzzing: Malicious payload 5</t>
+          <t>VUL: Dynamic code loading not permitted</t>
         </is>
       </c>
       <c r="D70" s="3" t="inlineStr">
@@ -2588,24 +2588,24 @@
         </is>
       </c>
       <c r="F70" s="3" t="n">
-        <v>20</v>
+        <v>1449</v>
       </c>
       <c r="G70" s="4" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" s="3" t="inlineStr">
         <is>
-          <t>TC-256</t>
+          <t>TC-M260</t>
         </is>
       </c>
       <c r="B71" s="4" t="inlineStr">
         <is>
-          <t>Vulnerability Testing</t>
+          <t>Extended Vulnerability</t>
         </is>
       </c>
       <c r="C71" s="4" t="inlineStr">
         <is>
-          <t>Header Fuzzing: Malicious payload 6</t>
+          <t>VUL: Backup flag disabled (no data in ADB backup)</t>
         </is>
       </c>
       <c r="D71" s="3" t="inlineStr">
@@ -2619,24 +2619,24 @@
         </is>
       </c>
       <c r="F71" s="3" t="n">
-        <v>20</v>
+        <v>1292</v>
       </c>
       <c r="G71" s="4" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" s="3" t="inlineStr">
         <is>
-          <t>TC-257</t>
+          <t>TC-M261</t>
         </is>
       </c>
       <c r="B72" s="4" t="inlineStr">
         <is>
-          <t>Vulnerability Testing</t>
+          <t>Extended Vulnerability</t>
         </is>
       </c>
       <c r="C72" s="4" t="inlineStr">
         <is>
-          <t>Header Fuzzing: Malicious payload 7</t>
+          <t>VUL: AllowBackup=false in manifest</t>
         </is>
       </c>
       <c r="D72" s="3" t="inlineStr">
@@ -2650,24 +2650,24 @@
         </is>
       </c>
       <c r="F72" s="3" t="n">
-        <v>20</v>
+        <v>120</v>
       </c>
       <c r="G72" s="4" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" s="3" t="inlineStr">
         <is>
-          <t>TC-258</t>
+          <t>TC-M262</t>
         </is>
       </c>
       <c r="B73" s="4" t="inlineStr">
         <is>
-          <t>Vulnerability Testing</t>
+          <t>Extended Vulnerability</t>
         </is>
       </c>
       <c r="C73" s="4" t="inlineStr">
         <is>
-          <t>Header Fuzzing: Malicious payload 8</t>
+          <t>VUL: Network security config restricts cleartext</t>
         </is>
       </c>
       <c r="D73" s="3" t="inlineStr">
@@ -2681,24 +2681,24 @@
         </is>
       </c>
       <c r="F73" s="3" t="n">
-        <v>20</v>
+        <v>468</v>
       </c>
       <c r="G73" s="4" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" s="3" t="inlineStr">
         <is>
-          <t>TC-259</t>
+          <t>TC-M263</t>
         </is>
       </c>
       <c r="B74" s="4" t="inlineStr">
         <is>
-          <t>Vulnerability Testing</t>
+          <t>Extended Vulnerability</t>
         </is>
       </c>
       <c r="C74" s="4" t="inlineStr">
         <is>
-          <t>Header Fuzzing: Malicious payload 9</t>
+          <t>VUL: Insecure direct object ref via donation ID blocked</t>
         </is>
       </c>
       <c r="D74" s="3" t="inlineStr">
@@ -2712,24 +2712,24 @@
         </is>
       </c>
       <c r="F74" s="3" t="n">
-        <v>20</v>
+        <v>138</v>
       </c>
       <c r="G74" s="4" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" s="3" t="inlineStr">
         <is>
-          <t>TC-260</t>
+          <t>TC-M264</t>
         </is>
       </c>
       <c r="B75" s="4" t="inlineStr">
         <is>
-          <t>Vulnerability Testing</t>
+          <t>Extended Vulnerability</t>
         </is>
       </c>
       <c r="C75" s="4" t="inlineStr">
         <is>
-          <t>Header Fuzzing: Malicious payload 10</t>
+          <t>VUL: Race condition on concurrent claim requests handled</t>
         </is>
       </c>
       <c r="D75" s="3" t="inlineStr">
@@ -2743,24 +2743,24 @@
         </is>
       </c>
       <c r="F75" s="3" t="n">
-        <v>20</v>
+        <v>1854</v>
       </c>
       <c r="G75" s="4" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" s="3" t="inlineStr">
         <is>
-          <t>TC-261</t>
+          <t>TC-M265</t>
         </is>
       </c>
       <c r="B76" s="4" t="inlineStr">
         <is>
-          <t>Vulnerability Testing</t>
+          <t>Extended Vulnerability</t>
         </is>
       </c>
       <c r="C76" s="4" t="inlineStr">
         <is>
-          <t>Injection: Payload variant 1 rejected gracefully</t>
+          <t>VUL: SSRF in address field does not trigger server-side fetch</t>
         </is>
       </c>
       <c r="D76" s="3" t="inlineStr">
@@ -2774,1249 +2774,9 @@
         </is>
       </c>
       <c r="F76" s="3" t="n">
-        <v>50</v>
+        <v>64</v>
       </c>
       <c r="G76" s="4" t="inlineStr"/>
-    </row>
-    <row r="77">
-      <c r="A77" s="3" t="inlineStr">
-        <is>
-          <t>TC-262</t>
-        </is>
-      </c>
-      <c r="B77" s="4" t="inlineStr">
-        <is>
-          <t>Vulnerability Testing</t>
-        </is>
-      </c>
-      <c r="C77" s="4" t="inlineStr">
-        <is>
-          <t>Injection: Payload variant 2 rejected gracefully</t>
-        </is>
-      </c>
-      <c r="D77" s="3" t="inlineStr">
-        <is>
-          <t>Security</t>
-        </is>
-      </c>
-      <c r="E77" s="5" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="F77" s="3" t="n">
-        <v>50</v>
-      </c>
-      <c r="G77" s="4" t="inlineStr"/>
-    </row>
-    <row r="78">
-      <c r="A78" s="3" t="inlineStr">
-        <is>
-          <t>TC-263</t>
-        </is>
-      </c>
-      <c r="B78" s="4" t="inlineStr">
-        <is>
-          <t>Vulnerability Testing</t>
-        </is>
-      </c>
-      <c r="C78" s="4" t="inlineStr">
-        <is>
-          <t>Injection: Payload variant 3 rejected gracefully</t>
-        </is>
-      </c>
-      <c r="D78" s="3" t="inlineStr">
-        <is>
-          <t>Security</t>
-        </is>
-      </c>
-      <c r="E78" s="5" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="F78" s="3" t="n">
-        <v>50</v>
-      </c>
-      <c r="G78" s="4" t="inlineStr"/>
-    </row>
-    <row r="79">
-      <c r="A79" s="3" t="inlineStr">
-        <is>
-          <t>TC-264</t>
-        </is>
-      </c>
-      <c r="B79" s="4" t="inlineStr">
-        <is>
-          <t>Vulnerability Testing</t>
-        </is>
-      </c>
-      <c r="C79" s="4" t="inlineStr">
-        <is>
-          <t>Injection: Payload variant 4 rejected gracefully</t>
-        </is>
-      </c>
-      <c r="D79" s="3" t="inlineStr">
-        <is>
-          <t>Security</t>
-        </is>
-      </c>
-      <c r="E79" s="5" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="F79" s="3" t="n">
-        <v>50</v>
-      </c>
-      <c r="G79" s="4" t="inlineStr"/>
-    </row>
-    <row r="80">
-      <c r="A80" s="3" t="inlineStr">
-        <is>
-          <t>TC-265</t>
-        </is>
-      </c>
-      <c r="B80" s="4" t="inlineStr">
-        <is>
-          <t>Vulnerability Testing</t>
-        </is>
-      </c>
-      <c r="C80" s="4" t="inlineStr">
-        <is>
-          <t>Injection: Payload variant 5 rejected gracefully</t>
-        </is>
-      </c>
-      <c r="D80" s="3" t="inlineStr">
-        <is>
-          <t>Security</t>
-        </is>
-      </c>
-      <c r="E80" s="5" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="F80" s="3" t="n">
-        <v>50</v>
-      </c>
-      <c r="G80" s="4" t="inlineStr"/>
-    </row>
-    <row r="81">
-      <c r="A81" s="3" t="inlineStr">
-        <is>
-          <t>TC-266</t>
-        </is>
-      </c>
-      <c r="B81" s="4" t="inlineStr">
-        <is>
-          <t>Vulnerability Testing</t>
-        </is>
-      </c>
-      <c r="C81" s="4" t="inlineStr">
-        <is>
-          <t>Injection: Payload variant 6 rejected gracefully</t>
-        </is>
-      </c>
-      <c r="D81" s="3" t="inlineStr">
-        <is>
-          <t>Security</t>
-        </is>
-      </c>
-      <c r="E81" s="5" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="F81" s="3" t="n">
-        <v>50</v>
-      </c>
-      <c r="G81" s="4" t="inlineStr"/>
-    </row>
-    <row r="82">
-      <c r="A82" s="3" t="inlineStr">
-        <is>
-          <t>TC-267</t>
-        </is>
-      </c>
-      <c r="B82" s="4" t="inlineStr">
-        <is>
-          <t>Vulnerability Testing</t>
-        </is>
-      </c>
-      <c r="C82" s="4" t="inlineStr">
-        <is>
-          <t>Injection: Payload variant 7 rejected gracefully</t>
-        </is>
-      </c>
-      <c r="D82" s="3" t="inlineStr">
-        <is>
-          <t>Security</t>
-        </is>
-      </c>
-      <c r="E82" s="5" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="F82" s="3" t="n">
-        <v>50</v>
-      </c>
-      <c r="G82" s="4" t="inlineStr"/>
-    </row>
-    <row r="83">
-      <c r="A83" s="3" t="inlineStr">
-        <is>
-          <t>TC-268</t>
-        </is>
-      </c>
-      <c r="B83" s="4" t="inlineStr">
-        <is>
-          <t>Vulnerability Testing</t>
-        </is>
-      </c>
-      <c r="C83" s="4" t="inlineStr">
-        <is>
-          <t>Injection: Payload variant 8 rejected gracefully</t>
-        </is>
-      </c>
-      <c r="D83" s="3" t="inlineStr">
-        <is>
-          <t>Security</t>
-        </is>
-      </c>
-      <c r="E83" s="5" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="F83" s="3" t="n">
-        <v>50</v>
-      </c>
-      <c r="G83" s="4" t="inlineStr"/>
-    </row>
-    <row r="84">
-      <c r="A84" s="3" t="inlineStr">
-        <is>
-          <t>TC-269</t>
-        </is>
-      </c>
-      <c r="B84" s="4" t="inlineStr">
-        <is>
-          <t>Vulnerability Testing</t>
-        </is>
-      </c>
-      <c r="C84" s="4" t="inlineStr">
-        <is>
-          <t>Injection: Payload variant 9 rejected gracefully</t>
-        </is>
-      </c>
-      <c r="D84" s="3" t="inlineStr">
-        <is>
-          <t>Security</t>
-        </is>
-      </c>
-      <c r="E84" s="5" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="F84" s="3" t="n">
-        <v>50</v>
-      </c>
-      <c r="G84" s="4" t="inlineStr"/>
-    </row>
-    <row r="85">
-      <c r="A85" s="3" t="inlineStr">
-        <is>
-          <t>TC-270</t>
-        </is>
-      </c>
-      <c r="B85" s="4" t="inlineStr">
-        <is>
-          <t>Vulnerability Testing</t>
-        </is>
-      </c>
-      <c r="C85" s="4" t="inlineStr">
-        <is>
-          <t>Injection: Payload variant 10 rejected gracefully</t>
-        </is>
-      </c>
-      <c r="D85" s="3" t="inlineStr">
-        <is>
-          <t>Security</t>
-        </is>
-      </c>
-      <c r="E85" s="5" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="F85" s="3" t="n">
-        <v>50</v>
-      </c>
-      <c r="G85" s="4" t="inlineStr"/>
-    </row>
-    <row r="86">
-      <c r="A86" s="3" t="inlineStr">
-        <is>
-          <t>TC-271</t>
-        </is>
-      </c>
-      <c r="B86" s="4" t="inlineStr">
-        <is>
-          <t>Vulnerability Testing</t>
-        </is>
-      </c>
-      <c r="C86" s="4" t="inlineStr">
-        <is>
-          <t>Boundary: Securely handled business logic flaw 1</t>
-        </is>
-      </c>
-      <c r="D86" s="3" t="inlineStr">
-        <is>
-          <t>Security</t>
-        </is>
-      </c>
-      <c r="E86" s="5" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="F86" s="3" t="n">
-        <v>35</v>
-      </c>
-      <c r="G86" s="4" t="inlineStr"/>
-    </row>
-    <row r="87">
-      <c r="A87" s="3" t="inlineStr">
-        <is>
-          <t>TC-272</t>
-        </is>
-      </c>
-      <c r="B87" s="4" t="inlineStr">
-        <is>
-          <t>Vulnerability Testing</t>
-        </is>
-      </c>
-      <c r="C87" s="4" t="inlineStr">
-        <is>
-          <t>Boundary: Securely handled business logic flaw 2</t>
-        </is>
-      </c>
-      <c r="D87" s="3" t="inlineStr">
-        <is>
-          <t>Security</t>
-        </is>
-      </c>
-      <c r="E87" s="5" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="F87" s="3" t="n">
-        <v>35</v>
-      </c>
-      <c r="G87" s="4" t="inlineStr"/>
-    </row>
-    <row r="88">
-      <c r="A88" s="3" t="inlineStr">
-        <is>
-          <t>TC-273</t>
-        </is>
-      </c>
-      <c r="B88" s="4" t="inlineStr">
-        <is>
-          <t>Vulnerability Testing</t>
-        </is>
-      </c>
-      <c r="C88" s="4" t="inlineStr">
-        <is>
-          <t>Boundary: Securely handled business logic flaw 3</t>
-        </is>
-      </c>
-      <c r="D88" s="3" t="inlineStr">
-        <is>
-          <t>Security</t>
-        </is>
-      </c>
-      <c r="E88" s="5" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="F88" s="3" t="n">
-        <v>35</v>
-      </c>
-      <c r="G88" s="4" t="inlineStr"/>
-    </row>
-    <row r="89">
-      <c r="A89" s="3" t="inlineStr">
-        <is>
-          <t>TC-274</t>
-        </is>
-      </c>
-      <c r="B89" s="4" t="inlineStr">
-        <is>
-          <t>Vulnerability Testing</t>
-        </is>
-      </c>
-      <c r="C89" s="4" t="inlineStr">
-        <is>
-          <t>Boundary: Securely handled business logic flaw 4</t>
-        </is>
-      </c>
-      <c r="D89" s="3" t="inlineStr">
-        <is>
-          <t>Security</t>
-        </is>
-      </c>
-      <c r="E89" s="5" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="F89" s="3" t="n">
-        <v>35</v>
-      </c>
-      <c r="G89" s="4" t="inlineStr"/>
-    </row>
-    <row r="90">
-      <c r="A90" s="3" t="inlineStr">
-        <is>
-          <t>TC-275</t>
-        </is>
-      </c>
-      <c r="B90" s="4" t="inlineStr">
-        <is>
-          <t>Vulnerability Testing</t>
-        </is>
-      </c>
-      <c r="C90" s="4" t="inlineStr">
-        <is>
-          <t>Boundary: Securely handled business logic flaw 5</t>
-        </is>
-      </c>
-      <c r="D90" s="3" t="inlineStr">
-        <is>
-          <t>Security</t>
-        </is>
-      </c>
-      <c r="E90" s="5" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="F90" s="3" t="n">
-        <v>35</v>
-      </c>
-      <c r="G90" s="4" t="inlineStr"/>
-    </row>
-    <row r="91">
-      <c r="A91" s="3" t="inlineStr">
-        <is>
-          <t>TC-276</t>
-        </is>
-      </c>
-      <c r="B91" s="4" t="inlineStr">
-        <is>
-          <t>Vulnerability Testing</t>
-        </is>
-      </c>
-      <c r="C91" s="4" t="inlineStr">
-        <is>
-          <t>Boundary: Securely handled business logic flaw 6</t>
-        </is>
-      </c>
-      <c r="D91" s="3" t="inlineStr">
-        <is>
-          <t>Security</t>
-        </is>
-      </c>
-      <c r="E91" s="5" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="F91" s="3" t="n">
-        <v>35</v>
-      </c>
-      <c r="G91" s="4" t="inlineStr"/>
-    </row>
-    <row r="92">
-      <c r="A92" s="3" t="inlineStr">
-        <is>
-          <t>TC-277</t>
-        </is>
-      </c>
-      <c r="B92" s="4" t="inlineStr">
-        <is>
-          <t>Vulnerability Testing</t>
-        </is>
-      </c>
-      <c r="C92" s="4" t="inlineStr">
-        <is>
-          <t>Boundary: Securely handled business logic flaw 7</t>
-        </is>
-      </c>
-      <c r="D92" s="3" t="inlineStr">
-        <is>
-          <t>Security</t>
-        </is>
-      </c>
-      <c r="E92" s="5" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="F92" s="3" t="n">
-        <v>35</v>
-      </c>
-      <c r="G92" s="4" t="inlineStr"/>
-    </row>
-    <row r="93">
-      <c r="A93" s="3" t="inlineStr">
-        <is>
-          <t>TC-278</t>
-        </is>
-      </c>
-      <c r="B93" s="4" t="inlineStr">
-        <is>
-          <t>Vulnerability Testing</t>
-        </is>
-      </c>
-      <c r="C93" s="4" t="inlineStr">
-        <is>
-          <t>Boundary: Securely handled business logic flaw 8</t>
-        </is>
-      </c>
-      <c r="D93" s="3" t="inlineStr">
-        <is>
-          <t>Security</t>
-        </is>
-      </c>
-      <c r="E93" s="5" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="F93" s="3" t="n">
-        <v>35</v>
-      </c>
-      <c r="G93" s="4" t="inlineStr"/>
-    </row>
-    <row r="94">
-      <c r="A94" s="3" t="inlineStr">
-        <is>
-          <t>TC-279</t>
-        </is>
-      </c>
-      <c r="B94" s="4" t="inlineStr">
-        <is>
-          <t>Vulnerability Testing</t>
-        </is>
-      </c>
-      <c r="C94" s="4" t="inlineStr">
-        <is>
-          <t>Boundary: Securely handled business logic flaw 9</t>
-        </is>
-      </c>
-      <c r="D94" s="3" t="inlineStr">
-        <is>
-          <t>Security</t>
-        </is>
-      </c>
-      <c r="E94" s="5" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="F94" s="3" t="n">
-        <v>35</v>
-      </c>
-      <c r="G94" s="4" t="inlineStr"/>
-    </row>
-    <row r="95">
-      <c r="A95" s="3" t="inlineStr">
-        <is>
-          <t>TC-280</t>
-        </is>
-      </c>
-      <c r="B95" s="4" t="inlineStr">
-        <is>
-          <t>Vulnerability Testing</t>
-        </is>
-      </c>
-      <c r="C95" s="4" t="inlineStr">
-        <is>
-          <t>Boundary: Securely handled business logic flaw 10</t>
-        </is>
-      </c>
-      <c r="D95" s="3" t="inlineStr">
-        <is>
-          <t>Security</t>
-        </is>
-      </c>
-      <c r="E95" s="5" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="F95" s="3" t="n">
-        <v>35</v>
-      </c>
-      <c r="G95" s="4" t="inlineStr"/>
-    </row>
-    <row r="96">
-      <c r="A96" s="3" t="inlineStr">
-        <is>
-          <t>TC-281</t>
-        </is>
-      </c>
-      <c r="B96" s="4" t="inlineStr">
-        <is>
-          <t>Vulnerability Testing</t>
-        </is>
-      </c>
-      <c r="C96" s="4" t="inlineStr">
-        <is>
-          <t>Boundary: Securely handled business logic flaw 11</t>
-        </is>
-      </c>
-      <c r="D96" s="3" t="inlineStr">
-        <is>
-          <t>Security</t>
-        </is>
-      </c>
-      <c r="E96" s="5" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="F96" s="3" t="n">
-        <v>35</v>
-      </c>
-      <c r="G96" s="4" t="inlineStr"/>
-    </row>
-    <row r="97">
-      <c r="A97" s="3" t="inlineStr">
-        <is>
-          <t>TC-282</t>
-        </is>
-      </c>
-      <c r="B97" s="4" t="inlineStr">
-        <is>
-          <t>Vulnerability Testing</t>
-        </is>
-      </c>
-      <c r="C97" s="4" t="inlineStr">
-        <is>
-          <t>Boundary: Securely handled business logic flaw 12</t>
-        </is>
-      </c>
-      <c r="D97" s="3" t="inlineStr">
-        <is>
-          <t>Security</t>
-        </is>
-      </c>
-      <c r="E97" s="5" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="F97" s="3" t="n">
-        <v>35</v>
-      </c>
-      <c r="G97" s="4" t="inlineStr"/>
-    </row>
-    <row r="98">
-      <c r="A98" s="3" t="inlineStr">
-        <is>
-          <t>TC-283</t>
-        </is>
-      </c>
-      <c r="B98" s="4" t="inlineStr">
-        <is>
-          <t>Vulnerability Testing</t>
-        </is>
-      </c>
-      <c r="C98" s="4" t="inlineStr">
-        <is>
-          <t>Boundary: Securely handled business logic flaw 13</t>
-        </is>
-      </c>
-      <c r="D98" s="3" t="inlineStr">
-        <is>
-          <t>Security</t>
-        </is>
-      </c>
-      <c r="E98" s="5" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="F98" s="3" t="n">
-        <v>35</v>
-      </c>
-      <c r="G98" s="4" t="inlineStr"/>
-    </row>
-    <row r="99">
-      <c r="A99" s="3" t="inlineStr">
-        <is>
-          <t>TC-284</t>
-        </is>
-      </c>
-      <c r="B99" s="4" t="inlineStr">
-        <is>
-          <t>Vulnerability Testing</t>
-        </is>
-      </c>
-      <c r="C99" s="4" t="inlineStr">
-        <is>
-          <t>Boundary: Securely handled business logic flaw 14</t>
-        </is>
-      </c>
-      <c r="D99" s="3" t="inlineStr">
-        <is>
-          <t>Security</t>
-        </is>
-      </c>
-      <c r="E99" s="5" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="F99" s="3" t="n">
-        <v>35</v>
-      </c>
-      <c r="G99" s="4" t="inlineStr"/>
-    </row>
-    <row r="100">
-      <c r="A100" s="3" t="inlineStr">
-        <is>
-          <t>TC-285</t>
-        </is>
-      </c>
-      <c r="B100" s="4" t="inlineStr">
-        <is>
-          <t>Vulnerability Testing</t>
-        </is>
-      </c>
-      <c r="C100" s="4" t="inlineStr">
-        <is>
-          <t>Boundary: Securely handled business logic flaw 15</t>
-        </is>
-      </c>
-      <c r="D100" s="3" t="inlineStr">
-        <is>
-          <t>Security</t>
-        </is>
-      </c>
-      <c r="E100" s="5" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="F100" s="3" t="n">
-        <v>35</v>
-      </c>
-      <c r="G100" s="4" t="inlineStr"/>
-    </row>
-    <row r="101">
-      <c r="A101" s="3" t="inlineStr">
-        <is>
-          <t>TC-M118</t>
-        </is>
-      </c>
-      <c r="B101" s="4" t="inlineStr">
-        <is>
-          <t>Vulnerability Testing</t>
-        </is>
-      </c>
-      <c r="C101" s="4" t="inlineStr">
-        <is>
-          <t>VUL: No JWT returns 401 on donations endpoint</t>
-        </is>
-      </c>
-      <c r="D101" s="3" t="inlineStr">
-        <is>
-          <t>Security</t>
-        </is>
-      </c>
-      <c r="E101" s="5" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="F101" s="3" t="n">
-        <v>13</v>
-      </c>
-      <c r="G101" s="4" t="inlineStr"/>
-    </row>
-    <row r="102">
-      <c r="A102" s="3" t="inlineStr">
-        <is>
-          <t>TC-M119</t>
-        </is>
-      </c>
-      <c r="B102" s="4" t="inlineStr">
-        <is>
-          <t>Vulnerability Testing</t>
-        </is>
-      </c>
-      <c r="C102" s="4" t="inlineStr">
-        <is>
-          <t>VUL: NGO cannot POST donation (RBAC 403)</t>
-        </is>
-      </c>
-      <c r="D102" s="3" t="inlineStr">
-        <is>
-          <t>Security</t>
-        </is>
-      </c>
-      <c r="E102" s="5" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="F102" s="3" t="n">
-        <v>204</v>
-      </c>
-      <c r="G102" s="4" t="inlineStr"/>
-    </row>
-    <row r="103">
-      <c r="A103" s="3" t="inlineStr">
-        <is>
-          <t>TC-M120</t>
-        </is>
-      </c>
-      <c r="B103" s="4" t="inlineStr">
-        <is>
-          <t>Vulnerability Testing</t>
-        </is>
-      </c>
-      <c r="C103" s="4" t="inlineStr">
-        <is>
-          <t>VUL: Donor cannot accept donations (RBAC 403/400)</t>
-        </is>
-      </c>
-      <c r="D103" s="3" t="inlineStr">
-        <is>
-          <t>Security</t>
-        </is>
-      </c>
-      <c r="E103" s="5" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="F103" s="3" t="n">
-        <v>223</v>
-      </c>
-      <c r="G103" s="4" t="inlineStr"/>
-    </row>
-    <row r="104">
-      <c r="A104" s="3" t="inlineStr">
-        <is>
-          <t>TC-M121</t>
-        </is>
-      </c>
-      <c r="B104" s="4" t="inlineStr">
-        <is>
-          <t>Vulnerability Testing</t>
-        </is>
-      </c>
-      <c r="C104" s="4" t="inlineStr">
-        <is>
-          <t>VUL: SQL injection in email does not cause 500</t>
-        </is>
-      </c>
-      <c r="D104" s="3" t="inlineStr">
-        <is>
-          <t>Security</t>
-        </is>
-      </c>
-      <c r="E104" s="5" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="F104" s="3" t="n">
-        <v>3</v>
-      </c>
-      <c r="G104" s="4" t="inlineStr"/>
-    </row>
-    <row r="105">
-      <c r="A105" s="3" t="inlineStr">
-        <is>
-          <t>TC-M122</t>
-        </is>
-      </c>
-      <c r="B105" s="4" t="inlineStr">
-        <is>
-          <t>Vulnerability Testing</t>
-        </is>
-      </c>
-      <c r="C105" s="4" t="inlineStr">
-        <is>
-          <t>VUL: XSS payload in signup - server responds without hanging</t>
-        </is>
-      </c>
-      <c r="D105" s="3" t="inlineStr">
-        <is>
-          <t>Security</t>
-        </is>
-      </c>
-      <c r="E105" s="5" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="F105" s="3" t="n">
-        <v>242</v>
-      </c>
-      <c r="G105" s="4" t="inlineStr"/>
-    </row>
-    <row r="106">
-      <c r="A106" s="3" t="inlineStr">
-        <is>
-          <t>TC-M123</t>
-        </is>
-      </c>
-      <c r="B106" s="4" t="inlineStr">
-        <is>
-          <t>Vulnerability Testing</t>
-        </is>
-      </c>
-      <c r="C106" s="4" t="inlineStr">
-        <is>
-          <t>VUL: Command injection in address field rejected gracefully</t>
-        </is>
-      </c>
-      <c r="D106" s="3" t="inlineStr">
-        <is>
-          <t>Security</t>
-        </is>
-      </c>
-      <c r="E106" s="5" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="F106" s="3" t="n">
-        <v>210</v>
-      </c>
-      <c r="G106" s="4" t="inlineStr"/>
-    </row>
-    <row r="107">
-      <c r="A107" s="3" t="inlineStr">
-        <is>
-          <t>TC-M124</t>
-        </is>
-      </c>
-      <c r="B107" s="4" t="inlineStr">
-        <is>
-          <t>Vulnerability Testing</t>
-        </is>
-      </c>
-      <c r="C107" s="4" t="inlineStr">
-        <is>
-          <t>VUL: Tampered JWT rejected with 401/422</t>
-        </is>
-      </c>
-      <c r="D107" s="3" t="inlineStr">
-        <is>
-          <t>Security</t>
-        </is>
-      </c>
-      <c r="E107" s="5" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="F107" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="G107" s="4" t="inlineStr"/>
-    </row>
-    <row r="108">
-      <c r="A108" s="3" t="inlineStr">
-        <is>
-          <t>TC-M125</t>
-        </is>
-      </c>
-      <c r="B108" s="4" t="inlineStr">
-        <is>
-          <t>Vulnerability Testing</t>
-        </is>
-      </c>
-      <c r="C108" s="4" t="inlineStr">
-        <is>
-          <t>VUL: Empty bearer token rejected</t>
-        </is>
-      </c>
-      <c r="D108" s="3" t="inlineStr">
-        <is>
-          <t>Security</t>
-        </is>
-      </c>
-      <c r="E108" s="5" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="F108" s="3" t="n">
-        <v>27</v>
-      </c>
-      <c r="G108" s="4" t="inlineStr"/>
-    </row>
-    <row r="109">
-      <c r="A109" s="3" t="inlineStr">
-        <is>
-          <t>TC-M126</t>
-        </is>
-      </c>
-      <c r="B109" s="4" t="inlineStr">
-        <is>
-          <t>Vulnerability Testing</t>
-        </is>
-      </c>
-      <c r="C109" s="4" t="inlineStr">
-        <is>
-          <t>VUL: Brute force - repeated wrong passwords all return 401</t>
-        </is>
-      </c>
-      <c r="D109" s="3" t="inlineStr">
-        <is>
-          <t>Security</t>
-        </is>
-      </c>
-      <c r="E109" s="5" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="F109" s="3" t="n">
-        <v>1555</v>
-      </c>
-      <c r="G109" s="4" t="inlineStr"/>
-    </row>
-    <row r="110">
-      <c r="A110" s="3" t="inlineStr">
-        <is>
-          <t>TC-M127</t>
-        </is>
-      </c>
-      <c r="B110" s="4" t="inlineStr">
-        <is>
-          <t>Vulnerability Testing</t>
-        </is>
-      </c>
-      <c r="C110" s="4" t="inlineStr">
-        <is>
-          <t>VUL: Server responds to malformed JSON without hanging</t>
-        </is>
-      </c>
-      <c r="D110" s="3" t="inlineStr">
-        <is>
-          <t>Security</t>
-        </is>
-      </c>
-      <c r="E110" s="5" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="F110" s="3" t="n">
-        <v>5</v>
-      </c>
-      <c r="G110" s="4" t="inlineStr"/>
-    </row>
-    <row r="111">
-      <c r="A111" s="3" t="inlineStr">
-        <is>
-          <t>TC-M128</t>
-        </is>
-      </c>
-      <c r="B111" s="4" t="inlineStr">
-        <is>
-          <t>Vulnerability Testing</t>
-        </is>
-      </c>
-      <c r="C111" s="4" t="inlineStr">
-        <is>
-          <t>VUL: Mass assignment - extra fields ignored in signup</t>
-        </is>
-      </c>
-      <c r="D111" s="3" t="inlineStr">
-        <is>
-          <t>Security</t>
-        </is>
-      </c>
-      <c r="E111" s="5" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="F111" s="3" t="n">
-        <v>236</v>
-      </c>
-      <c r="G111" s="4" t="inlineStr"/>
-    </row>
-    <row r="112">
-      <c r="A112" s="3" t="inlineStr">
-        <is>
-          <t>TC-M129</t>
-        </is>
-      </c>
-      <c r="B112" s="4" t="inlineStr">
-        <is>
-          <t>Vulnerability Testing</t>
-        </is>
-      </c>
-      <c r="C112" s="4" t="inlineStr">
-        <is>
-          <t>VUL: Password not returned in profile response</t>
-        </is>
-      </c>
-      <c r="D112" s="3" t="inlineStr">
-        <is>
-          <t>Security</t>
-        </is>
-      </c>
-      <c r="E112" s="5" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="F112" s="3" t="n">
-        <v>203</v>
-      </c>
-      <c r="G112" s="4" t="inlineStr"/>
-    </row>
-    <row r="113">
-      <c r="A113" s="3" t="inlineStr">
-        <is>
-          <t>TC-M130</t>
-        </is>
-      </c>
-      <c r="B113" s="4" t="inlineStr">
-        <is>
-          <t>Vulnerability Testing</t>
-        </is>
-      </c>
-      <c r="C113" s="4" t="inlineStr">
-        <is>
-          <t>VUL: JWT has proper 3-part structure</t>
-        </is>
-      </c>
-      <c r="D113" s="3" t="inlineStr">
-        <is>
-          <t>Security</t>
-        </is>
-      </c>
-      <c r="E113" s="5" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="F113" s="3" t="n">
-        <v>216</v>
-      </c>
-      <c r="G113" s="4" t="inlineStr"/>
-    </row>
-    <row r="114">
-      <c r="A114" s="3" t="inlineStr">
-        <is>
-          <t>TC-M131</t>
-        </is>
-      </c>
-      <c r="B114" s="4" t="inlineStr">
-        <is>
-          <t>Vulnerability Testing</t>
-        </is>
-      </c>
-      <c r="C114" s="4" t="inlineStr">
-        <is>
-          <t>VUL: Oversized payload in login does not crash server</t>
-        </is>
-      </c>
-      <c r="D114" s="3" t="inlineStr">
-        <is>
-          <t>Security</t>
-        </is>
-      </c>
-      <c r="E114" s="5" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="F114" s="3" t="n">
-        <v>3</v>
-      </c>
-      <c r="G114" s="4" t="inlineStr"/>
-    </row>
-    <row r="115">
-      <c r="A115" s="3" t="inlineStr">
-        <is>
-          <t>TC-M132</t>
-        </is>
-      </c>
-      <c r="B115" s="4" t="inlineStr">
-        <is>
-          <t>Vulnerability Testing</t>
-        </is>
-      </c>
-      <c r="C115" s="4" t="inlineStr">
-        <is>
-          <t>VUL: Unicode and null bytes in login handled safely</t>
-        </is>
-      </c>
-      <c r="D115" s="3" t="inlineStr">
-        <is>
-          <t>Security</t>
-        </is>
-      </c>
-      <c r="E115" s="5" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="F115" s="3" t="n">
-        <v>3</v>
-      </c>
-      <c r="G115" s="4" t="inlineStr"/>
-    </row>
-    <row r="116">
-      <c r="A116" s="3" t="inlineStr">
-        <is>
-          <t>TC-M133</t>
-        </is>
-      </c>
-      <c r="B116" s="4" t="inlineStr">
-        <is>
-          <t>Vulnerability Testing</t>
-        </is>
-      </c>
-      <c r="C116" s="4" t="inlineStr">
-        <is>
-          <t>VUL: Mobile app driver does not expose raw credentials in page source</t>
-        </is>
-      </c>
-      <c r="D116" s="3" t="inlineStr">
-        <is>
-          <t>Security</t>
-        </is>
-      </c>
-      <c r="E116" s="5" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="F116" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="G116" s="4" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -4059,7 +2819,7 @@
       </c>
       <c r="B2" s="7" t="inlineStr">
         <is>
-          <t>2026-06-14 21:34:59</t>
+          <t>2026-07-23 10:32:04</t>
         </is>
       </c>
     </row>
@@ -4070,7 +2830,7 @@
         </is>
       </c>
       <c r="B3" s="7" t="n">
-        <v>113</v>
+        <v>73</v>
       </c>
     </row>
     <row r="4">
@@ -4080,7 +2840,7 @@
         </is>
       </c>
       <c r="B4" s="7" t="n">
-        <v>113</v>
+        <v>73</v>
       </c>
     </row>
     <row r="5">

</xml_diff>